<commit_message>
Fixed society-table53-54 (labeled tables, visual and RDF data schemes)
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/society-table54.xlsx
+++ b/sources/table_normalization/xlsx/society-table54.xlsx
@@ -1162,7 +1162,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1178,12 +1178,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1254,7 +1248,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1288,20 +1282,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1314,7 +1294,18 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="5"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1871,56 +1862,56 @@
       <c r="W3" s="10"/>
     </row>
     <row r="4" spans="3:23">
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="13" t="s">
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="14"/>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="15"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="20"/>
+      <c r="T4" s="20"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="21"/>
     </row>
     <row r="5" spans="3:23">
       <c r="C5" s="4"/>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16" t="s">
+      <c r="E5" s="22"/>
+      <c r="F5" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16" t="s">
+      <c r="G5" s="22"/>
+      <c r="H5" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16" t="s">
+      <c r="I5" s="22"/>
+      <c r="J5" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16" t="s">
+      <c r="K5" s="22"/>
+      <c r="L5" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="M5" s="16"/>
+      <c r="M5" s="22"/>
       <c r="N5" s="5" t="s">
         <v>4</v>
       </c>
@@ -1944,69 +1935,69 @@
     </row>
     <row r="6" spans="3:23">
       <c r="C6" s="4"/>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="20" t="s">
+      <c r="H6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="20" t="s">
+      <c r="J6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K6" s="21" t="s">
+      <c r="K6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="L6" s="20" t="s">
+      <c r="L6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="21" t="s">
+      <c r="M6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="N6" s="20" t="s">
+      <c r="N6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="O6" s="21" t="s">
+      <c r="O6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="P6" s="20" t="s">
+      <c r="P6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="Q6" s="21" t="s">
+      <c r="Q6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="R6" s="20" t="s">
+      <c r="R6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="S6" s="21" t="s">
+      <c r="S6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="T6" s="20" t="s">
+      <c r="T6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="U6" s="21" t="s">
+      <c r="U6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="V6" s="20" t="s">
+      <c r="V6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="W6" s="21" t="s">
+      <c r="W6" s="15" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="3:23">
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="7" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -5107,7 +5098,7 @@
       <c r="W75" s="8"/>
     </row>
     <row r="76" spans="3:23">
-      <c r="C76" s="22" t="s">
+      <c r="C76" s="16" t="s">
         <v>283</v>
       </c>
       <c r="D76" s="3"/>
@@ -5132,7 +5123,7 @@
       <c r="W76" s="10"/>
     </row>
     <row r="77" spans="3:23">
-      <c r="C77" s="22" t="s">
+      <c r="C77" s="16" t="s">
         <v>284</v>
       </c>
       <c r="D77" s="3"/>

</xml_diff>